<commit_message>
codescan/tabtools: expand QA, update baselines, and add SSC release g...
</commit_message>
<xml_diff>
--- a/tabtools/qa/baseline/workbooks/comptab_sections.xlsx
+++ b/tabtools/qa/baseline/workbooks/comptab_sections.xlsx
@@ -3504,10 +3504,10 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="1.7109375" style="2" customWidth="true"/>
-    <col min="2" max="2" width="18.7109375" style="3" customWidth="true"/>
-    <col min="3" max="3" width="6.0859375" style="4" customWidth="true"/>
-    <col min="4" max="4" width="12.0859375" style="5" customWidth="true"/>
-    <col min="5" max="5" width="8.3671875" style="6" customWidth="true"/>
+    <col min="2" max="2" width="20.7109375" style="3" customWidth="true"/>
+    <col min="3" max="3" width="10.7109375" style="4" customWidth="true"/>
+    <col min="4" max="4" width="18.7109375" style="5" customWidth="true"/>
+    <col min="5" max="5" width="8.7109375" style="6" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="true" ht="30" customHeight="true">

</xml_diff>